<commit_message>
1:14 pm Monday, 3 August 2026 (IST)
</commit_message>
<xml_diff>
--- a/Current_Running.xlsx
+++ b/Current_Running.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akum1255\Desktop\Current Task Progress\Leaning Status\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akhil\OneDrive\Desktop\Home\Leaning-Status\Leaning-Status\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD96D19D-3FE0-4229-A300-8D1D5EB172CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE5C56F-5C4D-4C81-B4C9-4DDC6FBA267D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="791" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="756" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Java ☑" sheetId="1" r:id="rId1"/>
     <sheet name="Angular ☑" sheetId="2" r:id="rId2"/>
     <sheet name="SQL ☑" sheetId="3" r:id="rId3"/>
-    <sheet name="Project(Docker+Jenkins) ☑" sheetId="4" r:id="rId4"/>
+    <sheet name="Project(Docker+Jenkins+AWS) ☑" sheetId="4" r:id="rId4"/>
     <sheet name="Spring -RameshF" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -1169,21 +1169,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="29.1796875" customWidth="1"/>
-    <col min="3" max="3" width="25.36328125" customWidth="1"/>
-    <col min="4" max="4" width="30.453125" customWidth="1"/>
-    <col min="5" max="5" width="34.453125" customWidth="1"/>
-    <col min="6" max="6" width="25.1796875" customWidth="1"/>
-    <col min="7" max="7" width="35.453125" customWidth="1"/>
-    <col min="8" max="8" width="28.1796875" customWidth="1"/>
-    <col min="9" max="9" width="31.1796875" customWidth="1"/>
-    <col min="10" max="10" width="14.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.21875" customWidth="1"/>
+    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="4" max="4" width="30.44140625" customWidth="1"/>
+    <col min="5" max="5" width="34.44140625" customWidth="1"/>
+    <col min="6" max="6" width="25.21875" customWidth="1"/>
+    <col min="7" max="7" width="35.44140625" customWidth="1"/>
+    <col min="8" max="8" width="28.21875" customWidth="1"/>
+    <col min="9" max="9" width="31.21875" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>64</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>65</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>69</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>70</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>71</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
         <v>72</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
         <v>73</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>74</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
         <v>75</v>
       </c>
@@ -1383,7 +1383,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>76</v>
       </c>
@@ -1403,7 +1403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>77</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
         <v>78</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
         <v>79</v>
       </c>
@@ -1463,7 +1463,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
         <v>80</v>
       </c>
@@ -1483,7 +1483,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
         <v>81</v>
       </c>
@@ -1509,7 +1509,7 @@
       <c r="K16" s="20"/>
       <c r="L16" s="21"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1523,7 +1523,7 @@
       <c r="K17" s="12"/>
       <c r="L17" s="13"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7" t="s">
@@ -1547,21 +1547,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85DB43D5-BA6A-4D04-97DD-F9F9661A378E}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.81640625" customWidth="1"/>
-    <col min="2" max="2" width="23.36328125" customWidth="1"/>
-    <col min="3" max="3" width="27.08984375" customWidth="1"/>
-    <col min="4" max="4" width="30.453125" customWidth="1"/>
-    <col min="5" max="5" width="29.36328125" customWidth="1"/>
-    <col min="6" max="6" width="23.81640625" customWidth="1"/>
-    <col min="7" max="7" width="35.453125" customWidth="1"/>
-    <col min="8" max="8" width="28.1796875" customWidth="1"/>
-    <col min="9" max="9" width="31.1796875" customWidth="1"/>
-    <col min="10" max="10" width="14.90625" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" customWidth="1"/>
+    <col min="3" max="3" width="27.109375" customWidth="1"/>
+    <col min="4" max="4" width="30.44140625" customWidth="1"/>
+    <col min="5" max="5" width="29.33203125" customWidth="1"/>
+    <col min="6" max="6" width="23.77734375" customWidth="1"/>
+    <col min="7" max="7" width="35.44140625" customWidth="1"/>
+    <col min="8" max="8" width="28.21875" customWidth="1"/>
+    <col min="9" max="9" width="31.21875" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -1581,7 +1581,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
@@ -1621,7 +1621,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>16</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
         <v>21</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
         <v>26</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>31</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
         <v>33</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>34</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>37</v>
       </c>
@@ -1747,7 +1747,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
         <v>38</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
       <c r="B12" s="27"/>
       <c r="C12" s="4"/>
@@ -1773,7 +1773,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="24"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="17"/>
       <c r="B13" s="28"/>
       <c r="C13" s="7" t="s">
@@ -1787,7 +1787,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="18"/>
       <c r="B14" s="29"/>
       <c r="C14" s="9"/>
@@ -1795,7 +1795,7 @@
       <c r="E14" s="9"/>
       <c r="F14" s="10"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
         <v>44</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
         <v>45</v>
       </c>
@@ -1831,7 +1831,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="25" t="s">
         <v>50</v>
       </c>
@@ -1854,7 +1854,7 @@
       <c r="J17" s="12"/>
       <c r="K17" s="13"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="25" t="s">
         <v>55</v>
       </c>
@@ -1873,7 +1873,7 @@
       <c r="J18" s="12"/>
       <c r="K18" s="13"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="25" t="s">
         <v>56</v>
       </c>
@@ -1892,7 +1892,7 @@
       <c r="J19" s="12"/>
       <c r="K19" s="13"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="25" t="s">
         <v>57</v>
       </c>
@@ -1911,7 +1911,7 @@
       <c r="J20" s="12"/>
       <c r="K20" s="13"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="25" t="s">
         <v>58</v>
       </c>
@@ -1930,7 +1930,7 @@
       <c r="J21" s="12"/>
       <c r="K21" s="13"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="25" t="s">
         <v>59</v>
       </c>
@@ -1949,7 +1949,7 @@
       <c r="J22" s="12"/>
       <c r="K22" s="13"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="25" t="s">
         <v>60</v>
       </c>
@@ -1968,7 +1968,7 @@
       <c r="J23" s="12"/>
       <c r="K23" s="13"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="26" t="s">
         <v>61</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="24"/>
       <c r="C25" s="4"/>
@@ -1990,7 +1990,7 @@
       <c r="E25" s="4"/>
       <c r="F25" s="24"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
       <c r="B26" s="8"/>
       <c r="C26" s="7" t="s">
@@ -2012,21 +2012,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{399F2CC3-BD48-474A-BAE5-847D3E9516FF}">
   <dimension ref="A1:L15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.90625" customWidth="1"/>
-    <col min="2" max="2" width="22.6328125" customWidth="1"/>
-    <col min="3" max="3" width="27.81640625" customWidth="1"/>
-    <col min="4" max="4" width="30.453125" customWidth="1"/>
-    <col min="5" max="5" width="33.36328125" customWidth="1"/>
-    <col min="6" max="6" width="34.453125" customWidth="1"/>
-    <col min="7" max="7" width="35.453125" customWidth="1"/>
-    <col min="8" max="8" width="28.1796875" customWidth="1"/>
-    <col min="9" max="9" width="31.1796875" customWidth="1"/>
-    <col min="10" max="10" width="14.90625" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
+    <col min="3" max="3" width="27.77734375" customWidth="1"/>
+    <col min="4" max="4" width="30.44140625" customWidth="1"/>
+    <col min="5" max="5" width="33.33203125" customWidth="1"/>
+    <col min="6" max="6" width="34.44140625" customWidth="1"/>
+    <col min="7" max="7" width="35.44140625" customWidth="1"/>
+    <col min="8" max="8" width="28.21875" customWidth="1"/>
+    <col min="9" max="9" width="31.21875" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
         <v>95</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
         <v>96</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>97</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
         <v>98</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
         <v>99</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="15"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -2154,7 +2154,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="17"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7" t="s">
@@ -2170,7 +2170,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="18"/>
       <c r="B9" s="16"/>
       <c r="C9" s="9"/>
@@ -2178,7 +2178,7 @@
       <c r="E9" s="9"/>
       <c r="F9" s="10"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>115</v>
       </c>
@@ -2198,7 +2198,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
         <v>116</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
         <v>93</v>
       </c>
@@ -2244,7 +2244,7 @@
       <c r="K12" s="12"/>
       <c r="L12" s="13"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
         <v>94</v>
       </c>
@@ -2262,7 +2262,7 @@
       <c r="K13" s="12"/>
       <c r="L13" s="13"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -2270,7 +2270,7 @@
       <c r="E14" s="4"/>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7" t="s">
@@ -2294,21 +2294,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F5CCDB0-BC81-4945-8026-509DC19E37BE}">
   <dimension ref="A1:L60"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.90625" customWidth="1"/>
-    <col min="2" max="2" width="22.6328125" customWidth="1"/>
-    <col min="3" max="3" width="27.81640625" customWidth="1"/>
-    <col min="4" max="4" width="30.453125" customWidth="1"/>
-    <col min="5" max="5" width="33.36328125" customWidth="1"/>
-    <col min="6" max="6" width="34.453125" customWidth="1"/>
-    <col min="7" max="7" width="35.453125" customWidth="1"/>
-    <col min="8" max="8" width="28.1796875" customWidth="1"/>
-    <col min="9" max="9" width="31.1796875" customWidth="1"/>
-    <col min="10" max="10" width="14.90625" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
+    <col min="3" max="3" width="27.77734375" customWidth="1"/>
+    <col min="4" max="4" width="30.44140625" customWidth="1"/>
+    <col min="5" max="5" width="33.33203125" customWidth="1"/>
+    <col min="6" max="6" width="34.44140625" customWidth="1"/>
+    <col min="7" max="7" width="35.44140625" customWidth="1"/>
+    <col min="8" max="8" width="28.21875" customWidth="1"/>
+    <col min="9" max="9" width="31.21875" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>119</v>
       </c>
@@ -2338,7 +2338,7 @@
       <c r="E2" s="35"/>
       <c r="F2" s="35"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
         <v>120</v>
       </c>
@@ -2358,7 +2358,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>96</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="15"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -2386,7 +2386,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="17"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7" t="s">
@@ -2402,7 +2402,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="18"/>
       <c r="B7" s="16"/>
       <c r="C7" s="9"/>
@@ -2410,7 +2410,7 @@
       <c r="E7" s="9"/>
       <c r="F7" s="10"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>121</v>
       </c>
@@ -2420,7 +2420,7 @@
       <c r="E8" s="35"/>
       <c r="F8" s="35"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>124</v>
       </c>
@@ -2440,7 +2440,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>96</v>
       </c>
@@ -2466,7 +2466,7 @@
       <c r="K10" s="12"/>
       <c r="L10" s="13"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="15"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -2480,7 +2480,7 @@
       <c r="K11" s="12"/>
       <c r="L11" s="13"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="17"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7" t="s">
@@ -2496,7 +2496,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="36"/>
       <c r="B13" s="16"/>
       <c r="C13" s="9"/>
@@ -2504,7 +2504,7 @@
       <c r="E13" s="9"/>
       <c r="F13" s="10"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
         <v>122</v>
       </c>
@@ -2514,7 +2514,7 @@
       <c r="E14" s="35"/>
       <c r="F14" s="35"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
         <v>125</v>
       </c>
@@ -2534,7 +2534,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
         <v>96</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="15"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -2562,7 +2562,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="5"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="17"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7" t="s">
@@ -2578,7 +2578,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="36"/>
       <c r="B19" s="16"/>
       <c r="C19" s="9"/>
@@ -2586,7 +2586,7 @@
       <c r="E19" s="9"/>
       <c r="F19" s="10"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
         <v>123</v>
       </c>
@@ -2596,7 +2596,7 @@
       <c r="E20" s="35"/>
       <c r="F20" s="35"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="25" t="s">
         <v>120</v>
       </c>
@@ -2616,7 +2616,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="25" t="s">
         <v>96</v>
       </c>
@@ -2636,7 +2636,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -2644,7 +2644,7 @@
       <c r="E23" s="4"/>
       <c r="F23" s="5"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="17"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7" t="s">
@@ -2660,7 +2660,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="36"/>
       <c r="B25" s="16"/>
       <c r="C25" s="9"/>
@@ -2668,7 +2668,7 @@
       <c r="E25" s="9"/>
       <c r="F25" s="10"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="14" t="s">
         <v>138</v>
       </c>
@@ -2678,7 +2678,7 @@
       <c r="E26" s="35"/>
       <c r="F26" s="35"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="25" t="s">
         <v>126</v>
       </c>
@@ -2698,7 +2698,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="25" t="s">
         <v>96</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="15"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2726,7 +2726,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="5"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="17"/>
       <c r="B30" s="7"/>
       <c r="C30" s="7" t="s">
@@ -2742,7 +2742,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="36"/>
       <c r="B31" s="16"/>
       <c r="C31" s="9"/>
@@ -2750,7 +2750,7 @@
       <c r="E31" s="9"/>
       <c r="F31" s="10"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
         <v>139</v>
       </c>
@@ -2760,7 +2760,7 @@
       <c r="E32" s="35"/>
       <c r="F32" s="35"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="25" t="s">
         <v>127</v>
       </c>
@@ -2780,7 +2780,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="25" t="s">
         <v>96</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="15"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2808,7 +2808,7 @@
       <c r="E35" s="4"/>
       <c r="F35" s="5"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="17"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7" t="s">
@@ -2824,7 +2824,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="36"/>
       <c r="B37" s="16"/>
       <c r="C37" s="9"/>
@@ -2832,7 +2832,7 @@
       <c r="E37" s="9"/>
       <c r="F37" s="10"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="14" t="s">
         <v>140</v>
       </c>
@@ -2842,7 +2842,7 @@
       <c r="E38" s="35"/>
       <c r="F38" s="35"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="25" t="s">
         <v>128</v>
       </c>
@@ -2862,7 +2862,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="25" t="s">
         <v>96</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="15"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2890,7 +2890,7 @@
       <c r="E41" s="4"/>
       <c r="F41" s="5"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="17"/>
       <c r="B42" s="7"/>
       <c r="C42" s="7" t="s">
@@ -2906,7 +2906,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="36"/>
       <c r="B43" s="16"/>
       <c r="C43" s="9"/>
@@ -2914,7 +2914,7 @@
       <c r="E43" s="9"/>
       <c r="F43" s="10"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
         <v>141</v>
       </c>
@@ -2924,7 +2924,7 @@
       <c r="E44" s="35"/>
       <c r="F44" s="35"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="25" t="s">
         <v>129</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="25" t="s">
         <v>96</v>
       </c>
@@ -2964,7 +2964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="15"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -2972,7 +2972,7 @@
       <c r="E47" s="4"/>
       <c r="F47" s="5"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="6"/>
       <c r="B48" s="7"/>
       <c r="C48" s="7" t="s">
@@ -2988,7 +2988,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="36"/>
       <c r="B49" s="16"/>
       <c r="C49" s="9"/>
@@ -2996,7 +2996,7 @@
       <c r="E49" s="9"/>
       <c r="F49" s="10"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="14" t="s">
         <v>142</v>
       </c>
@@ -3006,7 +3006,7 @@
       <c r="E50" s="35"/>
       <c r="F50" s="35"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="25" t="s">
         <v>129</v>
       </c>
@@ -3026,7 +3026,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="25" t="s">
         <v>96</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="15"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3054,7 +3054,7 @@
       <c r="E53" s="4"/>
       <c r="F53" s="5"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="6"/>
       <c r="B54" s="7"/>
       <c r="C54" s="7" t="s">
@@ -3070,7 +3070,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="36"/>
       <c r="B55" s="16"/>
       <c r="C55" s="9"/>
@@ -3078,7 +3078,7 @@
       <c r="E55" s="9"/>
       <c r="F55" s="10"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="14" t="s">
         <v>143</v>
       </c>
@@ -3088,7 +3088,7 @@
       <c r="E56" s="35"/>
       <c r="F56" s="35"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="25" t="s">
         <v>129</v>
       </c>
@@ -3108,7 +3108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="25" t="s">
         <v>96</v>
       </c>
@@ -3128,7 +3128,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="15"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -3136,7 +3136,7 @@
       <c r="E59" s="4"/>
       <c r="F59" s="5"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="6"/>
       <c r="B60" s="7"/>
       <c r="C60" s="7" t="s">
@@ -3161,17 +3161,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9871143-4846-498A-9587-6847C2BB1359}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="81.6328125" customWidth="1"/>
-    <col min="2" max="2" width="21.6328125" customWidth="1"/>
-    <col min="3" max="3" width="25.1796875" customWidth="1"/>
-    <col min="4" max="4" width="26.90625" customWidth="1"/>
-    <col min="5" max="5" width="34.453125" customWidth="1"/>
-    <col min="6" max="6" width="13.6328125" customWidth="1"/>
+    <col min="1" max="1" width="81.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.21875" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" customWidth="1"/>
+    <col min="5" max="5" width="34.44140625" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>130</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>131</v>
       </c>
@@ -3231,7 +3231,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>132</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>133</v>
       </c>
@@ -3271,7 +3271,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>134</v>
       </c>
@@ -3291,7 +3291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
         <v>135</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
         <v>136</v>
       </c>
@@ -3331,7 +3331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>137</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
         <v>75</v>
       </c>
@@ -3371,7 +3371,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>76</v>
       </c>
@@ -3391,7 +3391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>77</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
         <v>78</v>
       </c>
@@ -3431,7 +3431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
         <v>79</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
         <v>80</v>
       </c>
@@ -3471,7 +3471,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
         <v>81</v>
       </c>
@@ -3491,7 +3491,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -3499,7 +3499,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="5"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7" t="s">

</xml_diff>

<commit_message>
2:09 am Saturday, 8 August 2026 (IST)
</commit_message>
<xml_diff>
--- a/Current_Running.xlsx
+++ b/Current_Running.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akhil\OneDrive\Desktop\Home\Leaning-Status\Leaning-Status\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akhil\OneDrive\Desktop\Home\Leaning-Status\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE5C56F-5C4D-4C81-B4C9-4DDC6FBA267D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69C87C3-4B86-4373-AE21-557648B7D854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="756" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="756" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Java ☑" sheetId="1" r:id="rId1"/>
@@ -1247,19 +1247,19 @@
       <c r="A4" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="40" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="42">
         <v>11</v>
       </c>
     </row>
@@ -1267,19 +1267,19 @@
       <c r="A5" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="32">
+      <c r="F5" s="42">
         <v>1</v>
       </c>
     </row>
@@ -1307,19 +1307,19 @@
       <c r="A7" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="42">
         <v>16</v>
       </c>
     </row>
@@ -1327,19 +1327,19 @@
       <c r="A8" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="E8" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="42">
         <v>1</v>
       </c>
     </row>
@@ -1347,19 +1347,19 @@
       <c r="A9" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="42">
         <v>1</v>
       </c>
     </row>

</xml_diff>